<commit_message>
Lab 2: web UI ticket generator
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="17256" windowHeight="5772" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Результаты" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,11 +414,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="19.21875" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-  </cols>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -464,15 +461,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Пётр</t>
+          <t>Иван</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-14 15:49:41</t>
+          <t>2026-09-17 00:05:10</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -494,15 +491,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Пётр</t>
+          <t>Иван</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-14 15:52:12</t>
+          <t>2026-09-17 00:05:19</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">

</xml_diff>